<commit_message>
dynamic add some fields and values
</commit_message>
<xml_diff>
--- a/public/Final_Results.xlsx
+++ b/public/Final_Results.xlsx
@@ -2,16 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="CampaignControlForm" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,24 +47,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -427,7 +422,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -526,10 +521,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:V8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="13" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13" bestFit="1" customWidth="1" min="1" max="13"/>
     <col width="13" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="13" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="13" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -542,6 +537,15 @@
     <col width="13" bestFit="1" customWidth="1" min="11" max="11"/>
     <col width="13" bestFit="1" customWidth="1" min="12" max="12"/>
     <col width="13" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="13" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="11.21875" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="24" bestFit="1" customWidth="1" min="16" max="19"/>
+    <col width="13" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="13" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="13" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="22.5546875" bestFit="1" customWidth="1" min="20" max="22"/>
+    <col width="13" bestFit="1" customWidth="1" min="21" max="21"/>
+    <col width="13" bestFit="1" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,22 +576,22 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>campaignStart</t>
+          <t>campaign_start</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>campaignEnd</t>
+          <t>campaign_end</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>preCampaignStart</t>
+          <t>pre_start</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>preCampaignEnd</t>
+          <t>pre_end</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -608,6 +612,51 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>outlierMethod</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ctrl_ratio</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales_metric</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>SEGMENT_CATEGORICAL_1</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>SEGMENT_CATEGORICAL_2</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>SEGMENT_CATEGORICAL_3</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>SEGMENT_CATEGORICAL_4</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>SEGMENT_NUMERICAL_1</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>SEGMENT_NUMERICAL_2</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>SEGMENT_NUMERICAL_3</t>
         </is>
       </c>
     </row>
@@ -672,6 +721,49 @@
           <t>2*SD</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -734,6 +826,49 @@
           <t>2*SD</t>
         </is>
       </c>
+      <c r="N3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -796,6 +931,49 @@
           <t>3*SD</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -818,7 +996,6 @@
           <t>imguse.jpeg</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-07-18</t>
@@ -857,6 +1034,327 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-19T13:05:09.993133</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-19T13:23:18.588598</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2*SD</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-19T15:09:58.604633</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>null</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
upload file functionality done
</commit_message>
<xml_diff>
--- a/public/Final_Results.xlsx
+++ b/public/Final_Results.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="1" max="13"/>
@@ -1273,7 +1273,6 @@
           <t>imguse.jpeg</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>2026-07-19</t>
@@ -1353,6 +1352,1301 @@
         </is>
       </c>
       <c r="V8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:36:54.776622</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Resume_updated (3).docx</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2*SD</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:38:02.396400</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>test.csv</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>meta.csv</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>mmx.csv</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2*SD</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:43:28.058974</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Resume_updated (5).docx</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-20T10:21:18.263111</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2*SD</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-20T11:05:31.674325</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-20T11:19:28.952867</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-20T11:37:30.419420</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>3*SD</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-20T11:53:21.450398</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-20T11:59:40.120134</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2*SD</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-20T12:07:12.566964</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-20T12:18:22.926879</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Traditional</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>/uploads/Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>/uploads/NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>3*SD</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-20T12:21:48.648710</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Synthetic</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>/uploads/Damonte.mp3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>/uploads/imguse.jpeg</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>/uploads/NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>null</t>
         </is>

</xml_diff>

<commit_message>
upload func done with api end point and text changes
</commit_message>
<xml_diff>
--- a/public/Final_Results.xlsx
+++ b/public/Final_Results.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="1" max="13"/>
@@ -2652,6 +2652,112 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:32:16.913255</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>/metadata/Senior Frontend Developer Questionnaire.xlsx</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>/metadata/NEW IMMIGRATION WEBSITE.xlsx</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Apis implementation and ui
</commit_message>
<xml_diff>
--- a/public/Final_Results.xlsx
+++ b/public/Final_Results.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="1" max="13"/>
@@ -2673,7 +2673,6 @@
           <t>/metadata/NEW IMMIGRATION WEBSITE.xlsx</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -2753,6 +2752,217 @@
         </is>
       </c>
       <c r="V21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-22T13:50:59.266360</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Strat_data.xlsx</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>strat_meta.xlsx</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>["SEGMENT_CATEGORICAL_1", "SEGMENT_CATEGORICAL_2"]</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>["SALES_1"]</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>1*SD</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-22T14:32:32.090183</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Stratification</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Strat_data.xlsx</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>strat_meta.xlsx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>["SEGMENT_CATEGORICAL_3", "SEGMENT_CATEGORICAL_4"]</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>["SALES_1"]</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>3*SD</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>null</t>
         </is>

</xml_diff>